<commit_message>
Actualizacion menu digital version estable
</commit_message>
<xml_diff>
--- a/BASE DE DATOS MENU COMIDAS RAPIDAS.xlsx
+++ b/BASE DE DATOS MENU COMIDAS RAPIDAS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TRABAJO DE GRADO 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TRABAJO DE GRADO 2\MENU_DIGITAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D03F25C1-C514-48FF-943B-E1D3E46F8557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1C2B72-6D72-4625-927E-F66C77BA648F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{03C40A3C-929C-4BBD-96F5-CD04AA93EF42}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="73">
   <si>
     <t>REFERENCIA</t>
   </si>
@@ -244,18 +244,6 @@
   </si>
   <si>
     <t>HIT PERSONAL</t>
-  </si>
-  <si>
-    <t>DOMICILIO</t>
-  </si>
-  <si>
-    <t>D0000</t>
-  </si>
-  <si>
-    <t>D2000</t>
-  </si>
-  <si>
-    <t>SIN DOMICILIO</t>
   </si>
 </sst>
 </file>
@@ -318,14 +306,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -1114,32 +1101,16 @@
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B35" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D35" s="5">
-        <v>2000</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>73</v>
-      </c>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="1"/>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B36" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D36" s="5">
-        <v>0</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>73</v>
-      </c>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>